<commit_message>
Avance de Orden de Compra
Ligar campos con tablas correspondiente
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/USUARIOS.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/USUARIOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maria Luisa Martinez\Documents\NetBeansProjects\OCXRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{725C1C65-51CB-4EE2-A6E4-68C49B181AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1F17B5-4740-45FB-8EA4-F545CE1E8165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F173C3BF-BF45-4085-9BA4-BD846F4D371B}"/>
+    <workbookView xWindow="4800" yWindow="2640" windowWidth="14400" windowHeight="8170" xr2:uid="{F173C3BF-BF45-4085-9BA4-BD846F4D371B}"/>
   </bookViews>
   <sheets>
     <sheet name="USUARIOS" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>USUARIO</t>
   </si>
@@ -66,6 +66,24 @@
   </si>
   <si>
     <t>AREA</t>
+  </si>
+  <si>
+    <t>Patron</t>
+  </si>
+  <si>
+    <t>Jefazo</t>
+  </si>
+  <si>
+    <t>María Luisa</t>
+  </si>
+  <si>
+    <t>Desarrollador</t>
+  </si>
+  <si>
+    <t>Adderly</t>
+  </si>
+  <si>
+    <t>Facturista</t>
   </si>
 </sst>
 </file>
@@ -464,6 +482,12 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -472,6 +496,12 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -479,6 +509,12 @@
       </c>
       <c r="B4" t="s">
         <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>